<commit_message>
Within min-max PC transformation.
</commit_message>
<xml_diff>
--- a/results/02_taxa_assemblage/AU-Sweeping/tables/k2_au_sweep_full.xlsx
+++ b/results/02_taxa_assemblage/AU-Sweeping/tables/k2_au_sweep_full.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:K32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,50 +436,45 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>actual_n</t>
+          <t>newly_entered_site</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>newly_entered_site</t>
+          <t>AU_C1</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>AU_C1</t>
+          <t>BP_C1</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>BP_C1</t>
+          <t>size_C1</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>size_C1</t>
+          <t>AU_C2</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>AU_C2</t>
+          <t>BP_C2</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>BP_C2</t>
+          <t>size_C2</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>size_C2</t>
+          <t>min_AU</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>min_AU</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>min_size</t>
         </is>
@@ -490,39 +485,36 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>35</v>
-      </c>
-      <c r="C2" t="n">
-        <v>35</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>SCR-17</t>
-        </is>
+        <v>40</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>SCR-06</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.9044</v>
       </c>
       <c r="E2" t="n">
-        <v>0.6248</v>
+        <v>0.0044</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0187</v>
+        <v>17</v>
       </c>
       <c r="G2" t="n">
-        <v>14</v>
+        <v>0.9522</v>
       </c>
       <c r="H2" t="n">
-        <v>0.8919</v>
+        <v>0.0139</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0399</v>
+        <v>23</v>
       </c>
       <c r="J2" t="n">
-        <v>21</v>
+        <v>0.9044</v>
       </c>
       <c r="K2" t="n">
-        <v>0.6248</v>
-      </c>
-      <c r="L2" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
@@ -530,39 +522,36 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>36</v>
-      </c>
-      <c r="C3" t="n">
-        <v>36</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>LSC-56</t>
-        </is>
+        <v>41</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>LSC-55</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.5891</v>
       </c>
       <c r="E3" t="n">
-        <v>0.6747</v>
+        <v>0.1244</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0197</v>
+        <v>34</v>
       </c>
       <c r="G3" t="n">
-        <v>14</v>
+        <v>0.6149</v>
       </c>
       <c r="H3" t="n">
-        <v>0.8943</v>
+        <v>0.1502</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0398</v>
+        <v>7</v>
       </c>
       <c r="J3" t="n">
-        <v>22</v>
+        <v>0.5891</v>
       </c>
       <c r="K3" t="n">
-        <v>0.6747</v>
-      </c>
-      <c r="L3" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -570,39 +559,36 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>37</v>
-      </c>
-      <c r="C4" t="n">
-        <v>37</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>SCR-01</t>
-        </is>
+        <v>42</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>DR-03</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.6217</v>
       </c>
       <c r="E4" t="n">
-        <v>0.6872</v>
+        <v>0.1229</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0193</v>
+        <v>35</v>
       </c>
       <c r="G4" t="n">
-        <v>14</v>
+        <v>0.6331</v>
       </c>
       <c r="H4" t="n">
-        <v>0.8996</v>
+        <v>0.1479</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0387</v>
+        <v>7</v>
       </c>
       <c r="J4" t="n">
-        <v>23</v>
+        <v>0.6217</v>
       </c>
       <c r="K4" t="n">
-        <v>0.6872</v>
-      </c>
-      <c r="L4" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -610,39 +596,36 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>38</v>
-      </c>
-      <c r="C5" t="n">
-        <v>38</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>SCR-14</t>
-        </is>
+        <v>43</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>LSC-43</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0.5833</v>
       </c>
       <c r="E5" t="n">
-        <v>0.7347</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0235</v>
+        <v>35</v>
       </c>
       <c r="G5" t="n">
-        <v>14</v>
+        <v>0.5709</v>
       </c>
       <c r="H5" t="n">
-        <v>0.8997000000000001</v>
+        <v>0.1045</v>
       </c>
       <c r="I5" t="n">
-        <v>0.0431</v>
+        <v>8</v>
       </c>
       <c r="J5" t="n">
-        <v>24</v>
+        <v>0.5709</v>
       </c>
       <c r="K5" t="n">
-        <v>0.7347</v>
-      </c>
-      <c r="L5" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
@@ -650,39 +633,36 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>39</v>
-      </c>
-      <c r="C6" t="n">
-        <v>39</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>DR-94</t>
-        </is>
+        <v>44</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>SCR-20</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.5931</v>
       </c>
       <c r="E6" t="n">
-        <v>0.3816</v>
+        <v>0.09180000000000001</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0058</v>
+        <v>36</v>
       </c>
       <c r="G6" t="n">
-        <v>15</v>
+        <v>0.5703</v>
       </c>
       <c r="H6" t="n">
-        <v>0.5172</v>
+        <v>0.1108</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0073</v>
+        <v>8</v>
       </c>
       <c r="J6" t="n">
-        <v>24</v>
+        <v>0.5703</v>
       </c>
       <c r="K6" t="n">
-        <v>0.3816</v>
-      </c>
-      <c r="L6" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -690,39 +670,36 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>40</v>
-      </c>
-      <c r="C7" t="n">
-        <v>40</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>SCR-06</t>
-        </is>
+        <v>45</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>DR-145</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0.5979</v>
       </c>
       <c r="E7" t="n">
-        <v>0.9044</v>
+        <v>0.0898</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0044</v>
+        <v>37</v>
       </c>
       <c r="G7" t="n">
-        <v>17</v>
+        <v>0.5769</v>
       </c>
       <c r="H7" t="n">
-        <v>0.9522</v>
+        <v>0.1107</v>
       </c>
       <c r="I7" t="n">
-        <v>0.0139</v>
+        <v>8</v>
       </c>
       <c r="J7" t="n">
-        <v>23</v>
+        <v>0.5769</v>
       </c>
       <c r="K7" t="n">
-        <v>0.9044</v>
-      </c>
-      <c r="L7" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
@@ -730,39 +707,36 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>41</v>
-      </c>
-      <c r="C8" t="n">
-        <v>41</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>LSC-55</t>
-        </is>
+        <v>46</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>DR-143</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0.5068</v>
       </c>
       <c r="E8" t="n">
-        <v>0.5891</v>
+        <v>0.0326</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1244</v>
+        <v>37</v>
       </c>
       <c r="G8" t="n">
-        <v>34</v>
+        <v>0.5615</v>
       </c>
       <c r="H8" t="n">
-        <v>0.6149</v>
+        <v>0.0397</v>
       </c>
       <c r="I8" t="n">
-        <v>0.1502</v>
+        <v>9</v>
       </c>
       <c r="J8" t="n">
-        <v>7</v>
+        <v>0.5068</v>
       </c>
       <c r="K8" t="n">
-        <v>0.5891</v>
-      </c>
-      <c r="L8" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
@@ -770,39 +744,36 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>42</v>
-      </c>
-      <c r="C9" t="n">
-        <v>42</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>DR-03</t>
-        </is>
+        <v>47</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>LSC-15</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0.5669</v>
       </c>
       <c r="E9" t="n">
-        <v>0.6217</v>
+        <v>0.0322</v>
       </c>
       <c r="F9" t="n">
-        <v>0.1229</v>
+        <v>9</v>
       </c>
       <c r="G9" t="n">
-        <v>35</v>
+        <v>0.5961</v>
       </c>
       <c r="H9" t="n">
-        <v>0.6331</v>
+        <v>0.0379</v>
       </c>
       <c r="I9" t="n">
-        <v>0.1479</v>
+        <v>38</v>
       </c>
       <c r="J9" t="n">
-        <v>7</v>
+        <v>0.5669</v>
       </c>
       <c r="K9" t="n">
-        <v>0.6217</v>
-      </c>
-      <c r="L9" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10">
@@ -810,39 +781,36 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>43</v>
-      </c>
-      <c r="C10" t="n">
-        <v>43</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>LSC-43</t>
-        </is>
+        <v>48</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>DR-125</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0.5581</v>
       </c>
       <c r="E10" t="n">
-        <v>0.5833</v>
+        <v>0.0431</v>
       </c>
       <c r="F10" t="n">
-        <v>0.08799999999999999</v>
+        <v>10</v>
       </c>
       <c r="G10" t="n">
-        <v>35</v>
+        <v>0.6304999999999999</v>
       </c>
       <c r="H10" t="n">
-        <v>0.5709</v>
+        <v>0.0491</v>
       </c>
       <c r="I10" t="n">
-        <v>0.1045</v>
+        <v>38</v>
       </c>
       <c r="J10" t="n">
-        <v>8</v>
+        <v>0.5581</v>
       </c>
       <c r="K10" t="n">
-        <v>0.5709</v>
-      </c>
-      <c r="L10" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
@@ -850,39 +818,36 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>44</v>
-      </c>
-      <c r="C11" t="n">
-        <v>44</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>SCR-20</t>
-        </is>
+        <v>49</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>SCR-09</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>0.5525</v>
       </c>
       <c r="E11" t="n">
-        <v>0.5931</v>
+        <v>0.0428</v>
       </c>
       <c r="F11" t="n">
-        <v>0.09180000000000001</v>
+        <v>10</v>
       </c>
       <c r="G11" t="n">
-        <v>36</v>
+        <v>0.623</v>
       </c>
       <c r="H11" t="n">
-        <v>0.5703</v>
+        <v>0.0488</v>
       </c>
       <c r="I11" t="n">
-        <v>0.1108</v>
+        <v>39</v>
       </c>
       <c r="J11" t="n">
-        <v>8</v>
+        <v>0.5525</v>
       </c>
       <c r="K11" t="n">
-        <v>0.5703</v>
-      </c>
-      <c r="L11" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -890,39 +855,36 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>45</v>
-      </c>
-      <c r="C12" t="n">
-        <v>45</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>DR-145</t>
-        </is>
+        <v>50</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>LSC-37</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>0.5893</v>
       </c>
       <c r="E12" t="n">
-        <v>0.5979</v>
+        <v>0.0421</v>
       </c>
       <c r="F12" t="n">
-        <v>0.0898</v>
+        <v>10</v>
       </c>
       <c r="G12" t="n">
-        <v>37</v>
+        <v>0.6595</v>
       </c>
       <c r="H12" t="n">
-        <v>0.5769</v>
+        <v>0.0495</v>
       </c>
       <c r="I12" t="n">
-        <v>0.1107</v>
+        <v>40</v>
       </c>
       <c r="J12" t="n">
-        <v>8</v>
+        <v>0.5893</v>
       </c>
       <c r="K12" t="n">
-        <v>0.5769</v>
-      </c>
-      <c r="L12" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
@@ -930,39 +892,36 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>46</v>
-      </c>
-      <c r="C13" t="n">
-        <v>46</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>DR-143</t>
-        </is>
+        <v>51</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>SCR-02</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>0.064</v>
       </c>
       <c r="E13" t="n">
-        <v>0.5068</v>
+        <v>0.064</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0326</v>
+        <v>16</v>
       </c>
       <c r="G13" t="n">
-        <v>37</v>
+        <v>0.046</v>
       </c>
       <c r="H13" t="n">
-        <v>0.5615</v>
+        <v>0.046</v>
       </c>
       <c r="I13" t="n">
-        <v>0.0397</v>
+        <v>35</v>
       </c>
       <c r="J13" t="n">
-        <v>9</v>
+        <v>0.046</v>
       </c>
       <c r="K13" t="n">
-        <v>0.5068</v>
-      </c>
-      <c r="L13" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14">
@@ -970,39 +929,36 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>47</v>
-      </c>
-      <c r="C14" t="n">
-        <v>47</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>LSC-15</t>
-        </is>
+        <v>52</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>LSC-07</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>0.064</v>
       </c>
       <c r="E14" t="n">
-        <v>0.5669</v>
+        <v>0.064</v>
       </c>
       <c r="F14" t="n">
-        <v>0.0322</v>
+        <v>17</v>
       </c>
       <c r="G14" t="n">
-        <v>9</v>
+        <v>0.076</v>
       </c>
       <c r="H14" t="n">
-        <v>0.5961</v>
+        <v>0.076</v>
       </c>
       <c r="I14" t="n">
-        <v>0.0379</v>
+        <v>35</v>
       </c>
       <c r="J14" t="n">
-        <v>38</v>
+        <v>0.064</v>
       </c>
       <c r="K14" t="n">
-        <v>0.5669</v>
-      </c>
-      <c r="L14" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15">
@@ -1010,39 +966,36 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>48</v>
-      </c>
-      <c r="C15" t="n">
-        <v>48</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>DR-125</t>
-        </is>
+        <v>53</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>DR-141</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>0.124</v>
       </c>
       <c r="E15" t="n">
-        <v>0.5581</v>
+        <v>0.124</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0431</v>
+        <v>14</v>
       </c>
       <c r="G15" t="n">
-        <v>10</v>
+        <v>0.2906</v>
       </c>
       <c r="H15" t="n">
-        <v>0.6304999999999999</v>
+        <v>0.0045</v>
       </c>
       <c r="I15" t="n">
-        <v>0.0491</v>
+        <v>39</v>
       </c>
       <c r="J15" t="n">
-        <v>38</v>
+        <v>0.124</v>
       </c>
       <c r="K15" t="n">
-        <v>0.5581</v>
-      </c>
-      <c r="L15" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16">
@@ -1050,39 +1003,36 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>49</v>
-      </c>
-      <c r="C16" t="n">
-        <v>49</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>SCR-09</t>
-        </is>
+        <v>54</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>DR-157</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>0.098</v>
       </c>
       <c r="E16" t="n">
-        <v>0.5525</v>
+        <v>0.098</v>
       </c>
       <c r="F16" t="n">
-        <v>0.0428</v>
+        <v>14</v>
       </c>
       <c r="G16" t="n">
-        <v>10</v>
+        <v>0.2906</v>
       </c>
       <c r="H16" t="n">
-        <v>0.623</v>
+        <v>0.0045</v>
       </c>
       <c r="I16" t="n">
-        <v>0.0488</v>
+        <v>40</v>
       </c>
       <c r="J16" t="n">
-        <v>39</v>
+        <v>0.098</v>
       </c>
       <c r="K16" t="n">
-        <v>0.5525</v>
-      </c>
-      <c r="L16" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17">
@@ -1090,39 +1040,36 @@
         <v>15</v>
       </c>
       <c r="B17" t="n">
-        <v>50</v>
-      </c>
-      <c r="C17" t="n">
-        <v>50</v>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>LSC-37</t>
-        </is>
+        <v>55</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>LSC-47</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>0.066</v>
       </c>
       <c r="E17" t="n">
-        <v>0.5893</v>
+        <v>0.066</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0421</v>
+        <v>14</v>
       </c>
       <c r="G17" t="n">
-        <v>10</v>
+        <v>0.052</v>
       </c>
       <c r="H17" t="n">
-        <v>0.6595</v>
+        <v>0.052</v>
       </c>
       <c r="I17" t="n">
-        <v>0.0495</v>
+        <v>41</v>
       </c>
       <c r="J17" t="n">
-        <v>40</v>
+        <v>0.052</v>
       </c>
       <c r="K17" t="n">
-        <v>0.5893</v>
-      </c>
-      <c r="L17" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18">
@@ -1130,39 +1077,36 @@
         <v>16</v>
       </c>
       <c r="B18" t="n">
-        <v>51</v>
-      </c>
-      <c r="C18" t="n">
-        <v>51</v>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>SCR-02</t>
-        </is>
+        <v>56</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>LSC-30</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>0.05</v>
       </c>
       <c r="E18" t="n">
-        <v>0.064</v>
+        <v>0.05</v>
       </c>
       <c r="F18" t="n">
-        <v>0.064</v>
+        <v>14</v>
       </c>
       <c r="G18" t="n">
-        <v>16</v>
+        <v>0.062</v>
       </c>
       <c r="H18" t="n">
-        <v>0.046</v>
+        <v>0.062</v>
       </c>
       <c r="I18" t="n">
-        <v>0.046</v>
+        <v>42</v>
       </c>
       <c r="J18" t="n">
-        <v>35</v>
+        <v>0.05</v>
       </c>
       <c r="K18" t="n">
-        <v>0.046</v>
-      </c>
-      <c r="L18" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19">
@@ -1170,39 +1114,36 @@
         <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>52</v>
-      </c>
-      <c r="C19" t="n">
-        <v>52</v>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>LSC-07</t>
-        </is>
+        <v>57</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>DR-156</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>0.08400000000000001</v>
       </c>
       <c r="E19" t="n">
-        <v>0.064</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="F19" t="n">
-        <v>0.064</v>
+        <v>13</v>
       </c>
       <c r="G19" t="n">
-        <v>17</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="H19" t="n">
-        <v>0.076</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="I19" t="n">
-        <v>0.076</v>
+        <v>44</v>
       </c>
       <c r="J19" t="n">
-        <v>35</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="K19" t="n">
-        <v>0.064</v>
-      </c>
-      <c r="L19" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20">
@@ -1210,39 +1151,36 @@
         <v>18</v>
       </c>
       <c r="B20" t="n">
-        <v>53</v>
-      </c>
-      <c r="C20" t="n">
-        <v>53</v>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>DR-141</t>
-        </is>
+        <v>58</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>LSC-32</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>0.1289</v>
       </c>
       <c r="E20" t="n">
-        <v>0.124</v>
+        <v>0.0039</v>
       </c>
       <c r="F20" t="n">
-        <v>0.124</v>
+        <v>13</v>
       </c>
       <c r="G20" t="n">
-        <v>14</v>
+        <v>0.1289</v>
       </c>
       <c r="H20" t="n">
-        <v>0.2906</v>
+        <v>0.0039</v>
       </c>
       <c r="I20" t="n">
-        <v>0.0045</v>
+        <v>45</v>
       </c>
       <c r="J20" t="n">
-        <v>39</v>
+        <v>0.1289</v>
       </c>
       <c r="K20" t="n">
-        <v>0.124</v>
-      </c>
-      <c r="L20" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="21">
@@ -1250,38 +1188,35 @@
         <v>19</v>
       </c>
       <c r="B21" t="n">
-        <v>54</v>
-      </c>
-      <c r="C21" t="n">
-        <v>54</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>DR-157</t>
-        </is>
+        <v>59</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>LSC-48</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>0.7663</v>
       </c>
       <c r="E21" t="n">
-        <v>0.098</v>
+        <v>0.0044</v>
       </c>
       <c r="F21" t="n">
-        <v>0.098</v>
+        <v>14</v>
       </c>
       <c r="G21" t="n">
-        <v>14</v>
+        <v>0.8563</v>
       </c>
       <c r="H21" t="n">
-        <v>0.2906</v>
+        <v>0.005</v>
       </c>
       <c r="I21" t="n">
-        <v>0.0045</v>
+        <v>45</v>
       </c>
       <c r="J21" t="n">
-        <v>40</v>
+        <v>0.7663</v>
       </c>
       <c r="K21" t="n">
-        <v>0.098</v>
-      </c>
-      <c r="L21" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1290,38 +1225,35 @@
         <v>20</v>
       </c>
       <c r="B22" t="n">
-        <v>55</v>
-      </c>
-      <c r="C22" t="n">
-        <v>55</v>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>LSC-47</t>
-        </is>
+        <v>60</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>LSC-31</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>0.4868</v>
       </c>
       <c r="E22" t="n">
-        <v>0.066</v>
+        <v>0.0035</v>
       </c>
       <c r="F22" t="n">
-        <v>0.066</v>
+        <v>14</v>
       </c>
       <c r="G22" t="n">
-        <v>14</v>
+        <v>0.4868</v>
       </c>
       <c r="H22" t="n">
-        <v>0.052</v>
+        <v>0.0035</v>
       </c>
       <c r="I22" t="n">
-        <v>0.052</v>
+        <v>46</v>
       </c>
       <c r="J22" t="n">
-        <v>41</v>
+        <v>0.4868</v>
       </c>
       <c r="K22" t="n">
-        <v>0.052</v>
-      </c>
-      <c r="L22" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1330,39 +1262,36 @@
         <v>21</v>
       </c>
       <c r="B23" t="n">
-        <v>56</v>
-      </c>
-      <c r="C23" t="n">
-        <v>56</v>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>LSC-30</t>
-        </is>
+        <v>61</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>DR-25</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>0.054</v>
       </c>
       <c r="E23" t="n">
-        <v>0.05</v>
+        <v>0.054</v>
       </c>
       <c r="F23" t="n">
-        <v>0.05</v>
+        <v>15</v>
       </c>
       <c r="G23" t="n">
-        <v>14</v>
+        <v>0.056</v>
       </c>
       <c r="H23" t="n">
-        <v>0.062</v>
+        <v>0.056</v>
       </c>
       <c r="I23" t="n">
-        <v>0.062</v>
+        <v>46</v>
       </c>
       <c r="J23" t="n">
-        <v>42</v>
+        <v>0.054</v>
       </c>
       <c r="K23" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="L23" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="24">
@@ -1370,39 +1299,36 @@
         <v>22</v>
       </c>
       <c r="B24" t="n">
-        <v>57</v>
-      </c>
-      <c r="C24" t="n">
-        <v>57</v>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>DR-156</t>
-        </is>
+        <v>62</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>LSC-28</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>0.058</v>
       </c>
       <c r="E24" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.058</v>
       </c>
       <c r="F24" t="n">
-        <v>0.08400000000000001</v>
+        <v>15</v>
       </c>
       <c r="G24" t="n">
-        <v>13</v>
+        <v>0.066</v>
       </c>
       <c r="H24" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.066</v>
       </c>
       <c r="I24" t="n">
-        <v>0.08400000000000001</v>
+        <v>47</v>
       </c>
       <c r="J24" t="n">
-        <v>44</v>
+        <v>0.058</v>
       </c>
       <c r="K24" t="n">
-        <v>0.08400000000000001</v>
-      </c>
-      <c r="L24" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25">
@@ -1410,39 +1336,36 @@
         <v>23</v>
       </c>
       <c r="B25" t="n">
-        <v>58</v>
-      </c>
-      <c r="C25" t="n">
-        <v>58</v>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>LSC-32</t>
-        </is>
+        <v>63</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>DR-110</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>0.4899</v>
       </c>
       <c r="E25" t="n">
-        <v>0.1289</v>
+        <v>0.0035</v>
       </c>
       <c r="F25" t="n">
-        <v>0.0039</v>
+        <v>15</v>
       </c>
       <c r="G25" t="n">
-        <v>13</v>
+        <v>0.4899</v>
       </c>
       <c r="H25" t="n">
-        <v>0.1289</v>
+        <v>0.0035</v>
       </c>
       <c r="I25" t="n">
-        <v>0.0039</v>
+        <v>48</v>
       </c>
       <c r="J25" t="n">
-        <v>45</v>
+        <v>0.4899</v>
       </c>
       <c r="K25" t="n">
-        <v>0.1289</v>
-      </c>
-      <c r="L25" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="26">
@@ -1450,39 +1373,36 @@
         <v>24</v>
       </c>
       <c r="B26" t="n">
-        <v>59</v>
-      </c>
-      <c r="C26" t="n">
-        <v>59</v>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>LSC-48</t>
-        </is>
+        <v>64</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>LSC-46</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>0.481</v>
       </c>
       <c r="E26" t="n">
-        <v>0.7663</v>
+        <v>0.0034</v>
       </c>
       <c r="F26" t="n">
-        <v>0.0044</v>
+        <v>16</v>
       </c>
       <c r="G26" t="n">
-        <v>14</v>
+        <v>0.481</v>
       </c>
       <c r="H26" t="n">
-        <v>0.8563</v>
+        <v>0.0034</v>
       </c>
       <c r="I26" t="n">
-        <v>0.005</v>
+        <v>48</v>
       </c>
       <c r="J26" t="n">
-        <v>45</v>
+        <v>0.481</v>
       </c>
       <c r="K26" t="n">
-        <v>0.7663</v>
-      </c>
-      <c r="L26" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="27">
@@ -1490,39 +1410,36 @@
         <v>25</v>
       </c>
       <c r="B27" t="n">
-        <v>60</v>
-      </c>
-      <c r="C27" t="n">
-        <v>60</v>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>LSC-31</t>
-        </is>
+        <v>65</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>LSC-35</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>0.5258</v>
       </c>
       <c r="E27" t="n">
-        <v>0.4868</v>
+        <v>0.0034</v>
       </c>
       <c r="F27" t="n">
-        <v>0.0035</v>
+        <v>16</v>
       </c>
       <c r="G27" t="n">
-        <v>14</v>
+        <v>0.5258</v>
       </c>
       <c r="H27" t="n">
-        <v>0.4868</v>
+        <v>0.0034</v>
       </c>
       <c r="I27" t="n">
-        <v>0.0035</v>
+        <v>49</v>
       </c>
       <c r="J27" t="n">
-        <v>46</v>
+        <v>0.5258</v>
       </c>
       <c r="K27" t="n">
-        <v>0.4868</v>
-      </c>
-      <c r="L27" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="28">
@@ -1530,39 +1447,36 @@
         <v>26</v>
       </c>
       <c r="B28" t="n">
-        <v>61</v>
-      </c>
-      <c r="C28" t="n">
-        <v>61</v>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>DR-25</t>
-        </is>
+        <v>66</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>LSC-29</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>0.5228</v>
       </c>
       <c r="E28" t="n">
-        <v>0.054</v>
+        <v>0.0034</v>
       </c>
       <c r="F28" t="n">
-        <v>0.054</v>
+        <v>16</v>
       </c>
       <c r="G28" t="n">
-        <v>15</v>
+        <v>0.5228</v>
       </c>
       <c r="H28" t="n">
-        <v>0.056</v>
+        <v>0.0034</v>
       </c>
       <c r="I28" t="n">
-        <v>0.056</v>
+        <v>50</v>
       </c>
       <c r="J28" t="n">
-        <v>46</v>
+        <v>0.5228</v>
       </c>
       <c r="K28" t="n">
-        <v>0.054</v>
-      </c>
-      <c r="L28" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="29">
@@ -1570,39 +1484,36 @@
         <v>27</v>
       </c>
       <c r="B29" t="n">
-        <v>62</v>
-      </c>
-      <c r="C29" t="n">
-        <v>62</v>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>LSC-28</t>
-        </is>
+        <v>67</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>SCR-12</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>0.5228</v>
       </c>
       <c r="E29" t="n">
-        <v>0.058</v>
+        <v>0.0034</v>
       </c>
       <c r="F29" t="n">
-        <v>0.058</v>
+        <v>17</v>
       </c>
       <c r="G29" t="n">
-        <v>15</v>
+        <v>0.5228</v>
       </c>
       <c r="H29" t="n">
-        <v>0.066</v>
+        <v>0.0034</v>
       </c>
       <c r="I29" t="n">
-        <v>0.066</v>
+        <v>50</v>
       </c>
       <c r="J29" t="n">
-        <v>47</v>
+        <v>0.5228</v>
       </c>
       <c r="K29" t="n">
-        <v>0.058</v>
-      </c>
-      <c r="L29" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="30">
@@ -1610,39 +1521,36 @@
         <v>28</v>
       </c>
       <c r="B30" t="n">
-        <v>63</v>
-      </c>
-      <c r="C30" t="n">
-        <v>63</v>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>DR-110</t>
-        </is>
+        <v>68</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>DR-71</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>0.028</v>
       </c>
       <c r="E30" t="n">
-        <v>0.4899</v>
+        <v>0.028</v>
       </c>
       <c r="F30" t="n">
-        <v>0.0035</v>
+        <v>19</v>
       </c>
       <c r="G30" t="n">
-        <v>15</v>
+        <v>0.026</v>
       </c>
       <c r="H30" t="n">
-        <v>0.4899</v>
+        <v>0.026</v>
       </c>
       <c r="I30" t="n">
-        <v>0.0035</v>
+        <v>49</v>
       </c>
       <c r="J30" t="n">
-        <v>48</v>
+        <v>0.026</v>
       </c>
       <c r="K30" t="n">
-        <v>0.4899</v>
-      </c>
-      <c r="L30" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="31">
@@ -1650,39 +1558,36 @@
         <v>29</v>
       </c>
       <c r="B31" t="n">
-        <v>64</v>
-      </c>
-      <c r="C31" t="n">
-        <v>64</v>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>LSC-46</t>
-        </is>
+        <v>69</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>DR-123</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>0.032</v>
       </c>
       <c r="E31" t="n">
-        <v>0.481</v>
+        <v>0.032</v>
       </c>
       <c r="F31" t="n">
-        <v>0.0034</v>
+        <v>20</v>
       </c>
       <c r="G31" t="n">
-        <v>16</v>
+        <v>0.03</v>
       </c>
       <c r="H31" t="n">
-        <v>0.481</v>
+        <v>0.03</v>
       </c>
       <c r="I31" t="n">
-        <v>0.0034</v>
+        <v>49</v>
       </c>
       <c r="J31" t="n">
-        <v>48</v>
+        <v>0.03</v>
       </c>
       <c r="K31" t="n">
-        <v>0.481</v>
-      </c>
-      <c r="L31" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="32">
@@ -1690,238 +1595,35 @@
         <v>30</v>
       </c>
       <c r="B32" t="n">
-        <v>65</v>
-      </c>
-      <c r="C32" t="n">
-        <v>65</v>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>LSC-35</t>
-        </is>
+        <v>70</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>DR-140</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>0.024</v>
       </c>
       <c r="E32" t="n">
-        <v>0.5258</v>
+        <v>0.024</v>
       </c>
       <c r="F32" t="n">
-        <v>0.0034</v>
+        <v>20</v>
       </c>
       <c r="G32" t="n">
-        <v>16</v>
+        <v>0.036</v>
       </c>
       <c r="H32" t="n">
-        <v>0.5258</v>
+        <v>0.036</v>
       </c>
       <c r="I32" t="n">
-        <v>0.0034</v>
+        <v>50</v>
       </c>
       <c r="J32" t="n">
-        <v>49</v>
+        <v>0.024</v>
       </c>
       <c r="K32" t="n">
-        <v>0.5258</v>
-      </c>
-      <c r="L32" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="1" t="n">
-        <v>31</v>
-      </c>
-      <c r="B33" t="n">
-        <v>66</v>
-      </c>
-      <c r="C33" t="n">
-        <v>66</v>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>LSC-29</t>
-        </is>
-      </c>
-      <c r="E33" t="n">
-        <v>0.5228</v>
-      </c>
-      <c r="F33" t="n">
-        <v>0.0034</v>
-      </c>
-      <c r="G33" t="n">
-        <v>16</v>
-      </c>
-      <c r="H33" t="n">
-        <v>0.5228</v>
-      </c>
-      <c r="I33" t="n">
-        <v>0.0034</v>
-      </c>
-      <c r="J33" t="n">
-        <v>50</v>
-      </c>
-      <c r="K33" t="n">
-        <v>0.5228</v>
-      </c>
-      <c r="L33" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="1" t="n">
-        <v>32</v>
-      </c>
-      <c r="B34" t="n">
-        <v>67</v>
-      </c>
-      <c r="C34" t="n">
-        <v>67</v>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>SCR-12</t>
-        </is>
-      </c>
-      <c r="E34" t="n">
-        <v>0.5228</v>
-      </c>
-      <c r="F34" t="n">
-        <v>0.0034</v>
-      </c>
-      <c r="G34" t="n">
-        <v>17</v>
-      </c>
-      <c r="H34" t="n">
-        <v>0.5228</v>
-      </c>
-      <c r="I34" t="n">
-        <v>0.0034</v>
-      </c>
-      <c r="J34" t="n">
-        <v>50</v>
-      </c>
-      <c r="K34" t="n">
-        <v>0.5228</v>
-      </c>
-      <c r="L34" t="n">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="1" t="n">
-        <v>33</v>
-      </c>
-      <c r="B35" t="n">
-        <v>68</v>
-      </c>
-      <c r="C35" t="n">
-        <v>68</v>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>DR-71</t>
-        </is>
-      </c>
-      <c r="E35" t="n">
-        <v>0.028</v>
-      </c>
-      <c r="F35" t="n">
-        <v>0.028</v>
-      </c>
-      <c r="G35" t="n">
-        <v>19</v>
-      </c>
-      <c r="H35" t="n">
-        <v>0.026</v>
-      </c>
-      <c r="I35" t="n">
-        <v>0.026</v>
-      </c>
-      <c r="J35" t="n">
-        <v>49</v>
-      </c>
-      <c r="K35" t="n">
-        <v>0.026</v>
-      </c>
-      <c r="L35" t="n">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="1" t="n">
-        <v>34</v>
-      </c>
-      <c r="B36" t="n">
-        <v>69</v>
-      </c>
-      <c r="C36" t="n">
-        <v>69</v>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>DR-123</t>
-        </is>
-      </c>
-      <c r="E36" t="n">
-        <v>0.032</v>
-      </c>
-      <c r="F36" t="n">
-        <v>0.032</v>
-      </c>
-      <c r="G36" t="n">
-        <v>20</v>
-      </c>
-      <c r="H36" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="I36" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="J36" t="n">
-        <v>49</v>
-      </c>
-      <c r="K36" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="L36" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="1" t="n">
-        <v>35</v>
-      </c>
-      <c r="B37" t="n">
-        <v>70</v>
-      </c>
-      <c r="C37" t="n">
-        <v>70</v>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>DR-140</t>
-        </is>
-      </c>
-      <c r="E37" t="n">
-        <v>0.024</v>
-      </c>
-      <c r="F37" t="n">
-        <v>0.024</v>
-      </c>
-      <c r="G37" t="n">
-        <v>20</v>
-      </c>
-      <c r="H37" t="n">
-        <v>0.036</v>
-      </c>
-      <c r="I37" t="n">
-        <v>0.036</v>
-      </c>
-      <c r="J37" t="n">
-        <v>50</v>
-      </c>
-      <c r="K37" t="n">
-        <v>0.024</v>
-      </c>
-      <c r="L37" t="n">
         <v>20</v>
       </c>
     </row>

</xml_diff>